<commit_message>
Not working at all
</commit_message>
<xml_diff>
--- a/app/config/tables/resultado/forms/resultado/resultado.xlsx
+++ b/app/config/tables/resultado/forms/resultado/resultado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\resultado\forms\resultado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5DC824C-6DF0-459D-A8F1-0B418F3872D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6227BAD-EFC0-4A82-B26E-7601632A9EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="3" r:id="rId1"/>
@@ -365,7 +365,7 @@
     <t>default</t>
   </si>
   <si>
-    <t>"200"</t>
+    <t>data('campo')==200</t>
   </si>
 </sst>
 </file>
@@ -991,7 +991,7 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>2022010601</v>
+        <v>2022022800</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Not working at all, no warnings, just poor odk-x code
</commit_message>
<xml_diff>
--- a/app/config/tables/resultado/forms/resultado/resultado.xlsx
+++ b/app/config/tables/resultado/forms/resultado/resultado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\resultado\forms\resultado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0EA450-119D-49CF-8CB7-3E72C3E08017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E85394-6988-4F3C-9CCB-606FEF30227F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="116">
   <si>
     <t>type</t>
   </si>
@@ -375,6 +375,12 @@
   </si>
   <si>
     <t>Somente en caso que é menor que 200</t>
+  </si>
+  <si>
+    <t>lab</t>
+  </si>
+  <si>
+    <t>Inicias de Laboratorista</t>
   </si>
 </sst>
 </file>
@@ -507,7 +513,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -539,6 +545,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1357,9 +1366,6 @@
       <c r="G15" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="M15" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D16" s="2" t="s">
@@ -1372,9 +1378,6 @@
       <c r="G16" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="M16" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
@@ -1383,7 +1386,16 @@
       <c r="E17" s="10"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E18" s="10"/>
+      <c r="D18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="17"/>
+      <c r="F18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D19" s="2" t="s">
@@ -1486,22 +1498,22 @@
       <c r="I39" s="10"/>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
       <c r="H40" s="15"/>
       <c r="I40" s="10"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
       <c r="H41" s="15"/>
       <c r="I41" s="10"/>
     </row>

</xml_diff>

<commit_message>
versao 2020030801 de inicio de estudo
</commit_message>
<xml_diff>
--- a/app/config/tables/resultado/forms/resultado/resultado.xlsx
+++ b/app/config/tables/resultado/forms/resultado/resultado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\resultado\forms\resultado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50A180A-4271-4CF9-A8ED-0C36C4D34AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EADB469-FAE6-4E24-B2EB-2CCEEF7A59C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-285" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="3" r:id="rId1"/>
@@ -1021,7 +1021,7 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>2022022800</v>
+        <v>2020030801</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>